<commit_message>
R84: deck todo em WPC (decisao do proprietario) com a conta de temperatura no modelo
Faixa seca da piscina e deck norte saem do porcelanato R11 e vao para o WPC
coextrudado claro; patio da churrasqueira fica em porcelanato; borda da
piscina inalterada. A verificacao de R59 sai do texto da prancha e entra em
externo.temperatura_superficie (dois pontos (H), linear no albedo), com
WPC_ALBEDO como hipotese do fabricante; a auditoria avisa a temperatura
estimada de cada zona descalca em vez de proibir. Prainha confirmada.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fkp4cnaZ7T35C1uJU37Vsp
</commit_message>
<xml_diff>
--- a/porto-real/out/PORTO_REAL_COTACAO.xlsx
+++ b/porto-real/out/PORTO_REAL_COTACAO.xlsx
@@ -1514,7 +1514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Residência unifamiliar em Light Steel Frame · Manaus/AM · 307.08 m² fechados · revisão R83</t>
+          <t>Residência unifamiliar em Light Steel Frame · Manaus/AM · 307.08 m² fechados · revisão R84</t>
         </is>
       </c>
     </row>
@@ -8446,7 +8446,7 @@
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>EXT-BLOCO</t>
+          <t>EXT-PISO2</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -8456,16 +8456,16 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
+          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E90" s="12" t="n">
-        <v>2750</v>
+        <v>50.4</v>
       </c>
       <c r="F90" s="13" t="n">
         <v>0</v>
@@ -8475,7 +8475,7 @@
         <v/>
       </c>
       <c r="H90" s="15" t="n">
-        <v>4.8</v>
+        <v>320</v>
       </c>
       <c r="I90" s="16">
         <f>G90*H90</f>
@@ -8522,7 +8522,7 @@
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO2</t>
+          <t>EXT-BLOCO</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -8532,16 +8532,16 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
+          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>un</t>
         </is>
       </c>
       <c r="E91" s="12" t="n">
-        <v>33.12</v>
+        <v>2750</v>
       </c>
       <c r="F91" s="13" t="n">
         <v>0</v>
@@ -8551,7 +8551,7 @@
         <v/>
       </c>
       <c r="H91" s="15" t="n">
-        <v>320</v>
+        <v>4.8</v>
       </c>
       <c r="I91" s="16">
         <f>G91*H91</f>
@@ -8598,7 +8598,7 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISC-EST</t>
+          <t>EXT-PISO1</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -8608,16 +8608,16 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Piscina: casca de concreto armado 150 mm</t>
+          <t>faixa seca da piscina: WPC coextrudado claro</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E92" s="12" t="n">
-        <v>4.57</v>
+        <v>24.3</v>
       </c>
       <c r="F92" s="13" t="n">
         <v>0</v>
@@ -8627,7 +8627,7 @@
         <v/>
       </c>
       <c r="H92" s="15" t="n">
-        <v>1450</v>
+        <v>320</v>
       </c>
       <c r="I92" s="16">
         <f>G92*H92</f>
@@ -8674,7 +8674,7 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO4</t>
+          <t>EXT-PISC-EST</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -8684,16 +8684,16 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>patio e deck descoberto: porcelanato externo claro R11</t>
+          <t>Piscina: casca de concreto armado 150 mm</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E93" s="12" t="n">
-        <v>43.2</v>
+        <v>4.57</v>
       </c>
       <c r="F93" s="13" t="n">
         <v>0</v>
@@ -8703,7 +8703,7 @@
         <v/>
       </c>
       <c r="H93" s="15" t="n">
-        <v>148</v>
+        <v>1450</v>
       </c>
       <c r="I93" s="16">
         <f>G93*H93</f>
@@ -9206,7 +9206,7 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO1</t>
+          <t>EXT-PISO4</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -9216,7 +9216,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>faixa seca da piscina: porcelanato externo claro R11</t>
+          <t>patio da churrasqueira: porcelanato externo claro R11</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
@@ -9225,7 +9225,7 @@
         </is>
       </c>
       <c r="E100" s="12" t="n">
-        <v>24.3</v>
+        <v>25.92</v>
       </c>
       <c r="F100" s="13" t="n">
         <v>0</v>
@@ -20923,7 +20923,7 @@
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>EXT-BLOCO</t>
+          <t>EXT-PISO2</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -20933,16 +20933,16 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
+          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E90" s="14" t="n">
-        <v>2750</v>
+        <v>50.4</v>
       </c>
       <c r="F90" s="11" t="inlineStr"/>
       <c r="G90" s="11" t="inlineStr"/>
@@ -20960,7 +20960,7 @@
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO2</t>
+          <t>EXT-BLOCO</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -20970,16 +20970,16 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
+          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>un</t>
         </is>
       </c>
       <c r="E91" s="14" t="n">
-        <v>33.12</v>
+        <v>2750</v>
       </c>
       <c r="F91" s="11" t="inlineStr"/>
       <c r="G91" s="11" t="inlineStr"/>
@@ -20997,7 +20997,7 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISC-EST</t>
+          <t>EXT-PISO1</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -21007,16 +21007,16 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Piscina: casca de concreto armado 150 mm</t>
+          <t>faixa seca da piscina: WPC coextrudado claro</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E92" s="14" t="n">
-        <v>4.57</v>
+        <v>24.3</v>
       </c>
       <c r="F92" s="11" t="inlineStr"/>
       <c r="G92" s="11" t="inlineStr"/>
@@ -21034,7 +21034,7 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO4</t>
+          <t>EXT-PISC-EST</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -21044,16 +21044,16 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>patio e deck descoberto: porcelanato externo claro R11</t>
+          <t>Piscina: casca de concreto armado 150 mm</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E93" s="14" t="n">
-        <v>43.2</v>
+        <v>4.57</v>
       </c>
       <c r="F93" s="11" t="inlineStr"/>
       <c r="G93" s="11" t="inlineStr"/>
@@ -21293,7 +21293,7 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO1</t>
+          <t>EXT-PISO4</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>faixa seca da piscina: porcelanato externo claro R11</t>
+          <t>patio da churrasqueira: porcelanato externo claro R11</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
@@ -21312,7 +21312,7 @@
         </is>
       </c>
       <c r="E100" s="14" t="n">
-        <v>24.3</v>
+        <v>25.92</v>
       </c>
       <c r="F100" s="11" t="inlineStr"/>
       <c r="G100" s="11" t="inlineStr"/>

</xml_diff>

<commit_message>
R85: deck volta ao porcelanato (decisao desfeita pelo proprietario); a conta de temperatura fica e passa a ser derivada
A faixa seca da piscina e o deck norte voltam ao porcelanato claro R11; o WPC
recua para o deck coberto e a varanda gourmet, como antes de R84. O BOM volta
a R$ 1.082.125,72, o valor de R83.

O que R84 trouxe para dentro do modelo permanece e melhora: em
externo.temperatura_por_zona, "ao sol" deixa de ser palavra no nome da zona e
passa a ser derivado de Amb.coberto. A regra de R59 (WPC so onde nao bate sol)
deixa de ser comentario e vira conferencia — hoje silenciosa, e volta a
disparar se alguem trocar o material de uma zona descoberta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fkp4cnaZ7T35C1uJU37Vsp
</commit_message>
<xml_diff>
--- a/porto-real/out/PORTO_REAL_COTACAO.xlsx
+++ b/porto-real/out/PORTO_REAL_COTACAO.xlsx
@@ -1514,7 +1514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Residência unifamiliar em Light Steel Frame · Manaus/AM · 307.08 m² fechados · revisão R84</t>
+          <t>Residência unifamiliar em Light Steel Frame · Manaus/AM · 307.08 m² fechados · revisão R85</t>
         </is>
       </c>
     </row>
@@ -8446,7 +8446,7 @@
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO2</t>
+          <t>EXT-BLOCO</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -8456,16 +8456,16 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
+          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>un</t>
         </is>
       </c>
       <c r="E90" s="12" t="n">
-        <v>50.4</v>
+        <v>2750</v>
       </c>
       <c r="F90" s="13" t="n">
         <v>0</v>
@@ -8475,7 +8475,7 @@
         <v/>
       </c>
       <c r="H90" s="15" t="n">
-        <v>320</v>
+        <v>4.8</v>
       </c>
       <c r="I90" s="16">
         <f>G90*H90</f>
@@ -8522,7 +8522,7 @@
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>EXT-BLOCO</t>
+          <t>EXT-PISO2</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -8532,16 +8532,16 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
+          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E91" s="12" t="n">
-        <v>2750</v>
+        <v>33.12</v>
       </c>
       <c r="F91" s="13" t="n">
         <v>0</v>
@@ -8551,7 +8551,7 @@
         <v/>
       </c>
       <c r="H91" s="15" t="n">
-        <v>4.8</v>
+        <v>320</v>
       </c>
       <c r="I91" s="16">
         <f>G91*H91</f>
@@ -8598,7 +8598,7 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO1</t>
+          <t>EXT-PISC-EST</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -8608,16 +8608,16 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>faixa seca da piscina: WPC coextrudado claro</t>
+          <t>Piscina: casca de concreto armado 150 mm</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E92" s="12" t="n">
-        <v>24.3</v>
+        <v>4.57</v>
       </c>
       <c r="F92" s="13" t="n">
         <v>0</v>
@@ -8627,7 +8627,7 @@
         <v/>
       </c>
       <c r="H92" s="15" t="n">
-        <v>320</v>
+        <v>1450</v>
       </c>
       <c r="I92" s="16">
         <f>G92*H92</f>
@@ -8674,7 +8674,7 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISC-EST</t>
+          <t>EXT-PISO4</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -8684,16 +8684,16 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Piscina: casca de concreto armado 150 mm</t>
+          <t>patio e deck descoberto: porcelanato externo claro R11</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E93" s="12" t="n">
-        <v>4.57</v>
+        <v>43.2</v>
       </c>
       <c r="F93" s="13" t="n">
         <v>0</v>
@@ -8703,7 +8703,7 @@
         <v/>
       </c>
       <c r="H93" s="15" t="n">
-        <v>1450</v>
+        <v>148</v>
       </c>
       <c r="I93" s="16">
         <f>G93*H93</f>
@@ -9206,7 +9206,7 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO4</t>
+          <t>EXT-PISO1</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -9216,7 +9216,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>patio da churrasqueira: porcelanato externo claro R11</t>
+          <t>faixa seca da piscina: porcelanato externo claro R11</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
@@ -9225,7 +9225,7 @@
         </is>
       </c>
       <c r="E100" s="12" t="n">
-        <v>25.92</v>
+        <v>24.3</v>
       </c>
       <c r="F100" s="13" t="n">
         <v>0</v>
@@ -20923,7 +20923,7 @@
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO2</t>
+          <t>EXT-BLOCO</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -20933,16 +20933,16 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
+          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>un</t>
         </is>
       </c>
       <c r="E90" s="14" t="n">
-        <v>50.4</v>
+        <v>2750</v>
       </c>
       <c r="F90" s="11" t="inlineStr"/>
       <c r="G90" s="11" t="inlineStr"/>
@@ -20960,7 +20960,7 @@
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>EXT-BLOCO</t>
+          <t>EXT-PISO2</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -20970,16 +20970,16 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Muro: bloco de concreto estrutural 14 x 19 x 39 ap</t>
+          <t>lounge e circulacao do deck: WPC coextrudado claro</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E91" s="14" t="n">
-        <v>2750</v>
+        <v>33.12</v>
       </c>
       <c r="F91" s="11" t="inlineStr"/>
       <c r="G91" s="11" t="inlineStr"/>
@@ -20997,7 +20997,7 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO1</t>
+          <t>EXT-PISC-EST</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -21007,16 +21007,16 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>faixa seca da piscina: WPC coextrudado claro</t>
+          <t>Piscina: casca de concreto armado 150 mm</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E92" s="14" t="n">
-        <v>24.3</v>
+        <v>4.57</v>
       </c>
       <c r="F92" s="11" t="inlineStr"/>
       <c r="G92" s="11" t="inlineStr"/>
@@ -21034,7 +21034,7 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISC-EST</t>
+          <t>EXT-PISO4</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -21044,16 +21044,16 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Piscina: casca de concreto armado 150 mm</t>
+          <t>patio e deck descoberto: porcelanato externo claro R11</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E93" s="14" t="n">
-        <v>4.57</v>
+        <v>43.2</v>
       </c>
       <c r="F93" s="11" t="inlineStr"/>
       <c r="G93" s="11" t="inlineStr"/>
@@ -21293,7 +21293,7 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>EXT-PISO4</t>
+          <t>EXT-PISO1</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>patio da churrasqueira: porcelanato externo claro R11</t>
+          <t>faixa seca da piscina: porcelanato externo claro R11</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr">
@@ -21312,7 +21312,7 @@
         </is>
       </c>
       <c r="E100" s="14" t="n">
-        <v>25.92</v>
+        <v>24.3</v>
       </c>
       <c r="F100" s="11" t="inlineStr"/>
       <c r="G100" s="11" t="inlineStr"/>

</xml_diff>